<commit_message>
Update Venteliste Parkering.xlsx from OneDrive
</commit_message>
<xml_diff>
--- a/Venteliste Parkering.xlsx
+++ b/Venteliste Parkering.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30621"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="888" documentId="11_924805B546FA86936262E6F9983E8C1851038381" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C8956B5-8139-423A-BB74-C95A578E969D}"/>
+  <xr:revisionPtr revIDLastSave="891" documentId="11_924805B546FA86936262E6F9983E8C1851038381" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF055A83-4BCE-4187-A0BB-AF399C5637AA}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2868,8 +2868,8 @@
         <f>D5&amp;" "&amp;E5&amp;", "&amp;F5&amp;"."&amp;G5</f>
         <v>Vigerslevvej 148, 1.tv</v>
       </c>
-      <c r="B5">
-        <v>0</v>
+      <c r="B5" s="7">
+        <v>46326</v>
       </c>
       <c r="C5">
         <v>10</v>

</xml_diff>